<commit_message>
Mk14 EBR aims through a 4x scope, and carrying a crate no longer slows you down
The Weapons tab has a new Scope magnification column (4 for the Mk14 EBR; empty = iron
sights). Aiming with a scoped weapon shows the scope view with slower look and slight drift.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CMHq89Xaygpa78Rxcwy3Lr
</commit_message>
<xml_diff>
--- a/data/Game Data.xlsx
+++ b/data/Game Data.xlsx
@@ -908,15 +908,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B3:Q11"/>
+  <dimension ref="B3:R11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.59765625" customWidth="1"/>
     <col min="2" max="14" width="15.59765625" customWidth="1"/>
     <col min="15" max="17" width="13" customWidth="1"/>
+    <col min="18" max="18" width="15.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:17" ht="57" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:18" ht="57" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B3" s="1" t="s">
         <v>17</v>
       </c>
@@ -964,6 +965,11 @@
       </c>
       <c r="Q3" s="1" t="s">
         <v>32</v>
+      </c>
+      <c r="R3" s="1" t="inlineStr">
+        <is>
+          <t>Scope magnification (empty = iron sights)</t>
+        </is>
       </c>
     </row>
     <row r="4" spans="2:17" x14ac:dyDescent="0.45">
@@ -1224,7 +1230,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="9" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B9" s="2" t="s">
         <v>47</v>
       </c>
@@ -1274,6 +1280,9 @@
       </c>
       <c r="Q9" s="3">
         <v>0.6</v>
+      </c>
+      <c r="R9" s="3">
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="2:17" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
Armour now protects against rockets and grenades; fuel tank blasts toned back
The RPG-7 and RGD-5 do 50 armour damage, so more than 50 armour survives a
direct hit (with 0, armour made you immune to explosions). Fuel tank blasts
are as strong as before the RPG got stronger.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CMHq89Xaygpa78Rxcwy3Lr
</commit_message>
<xml_diff>
--- a/data/Game Data.xlsx
+++ b/data/Game Data.xlsx
@@ -1481,7 +1481,7 @@
         <v>100</v>
       </c>
       <c r="G13" s="3">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H13" s="3">
         <v>50</v>
@@ -1532,7 +1532,7 @@
         <v>100</v>
       </c>
       <c r="G14" s="3">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H14" s="3">
         <v>100</v>

</xml_diff>

<commit_message>
New: automatic turret from the level 3 ammunition supply
Each player can take one turret from a level 3 ammunition supply, carry it
(no shooting), see where it will go (green or red) and DROP it; PICK UP
TURRET moves it again. It fires 5.56 bursts at 1,200 rounds a minute at
enemies it sees or hears; enemies fight it like a player. Destroyed, it
drops nothing and the supply hands out a new one. Its numbers are on the
new Allies tab and the Weapons tab's Turret row. Model: M134 minigun on a
tripod, from its reference sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CMHq89Xaygpa78Rxcwy3Lr
</commit_message>
<xml_diff>
--- a/data/Game Data.xlsx
+++ b/data/Game Data.xlsx
@@ -15,6 +15,7 @@
   <sheets>
     <sheet name="Enemies" sheetId="1" r:id="rId1"/>
     <sheet name="Weapons" sheetId="2" r:id="rId2"/>
+    <sheet name="Allies" sheetId="3" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1567,22 +1568,56 @@
       <c r="R14" s="3"/>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.45">
-      <c r="B15" s="2"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="3"/>
-      <c r="P15" s="3"/>
-      <c r="Q15" s="3"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Turret</t>
+        </is>
+      </c>
+      <c r="C15" s="3">
+        <v>100</v>
+      </c>
+      <c r="D15" s="3">
+        <v>100</v>
+      </c>
+      <c r="E15" s="3">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3">
+        <v>20</v>
+      </c>
+      <c r="G15" s="3">
+        <v>20</v>
+      </c>
+      <c r="H15" s="3">
+        <v>0</v>
+      </c>
+      <c r="I15" s="3">
+        <v>0</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="K15" s="3">
+        <v>1200</v>
+      </c>
+      <c r="L15" s="3">
+        <v>0</v>
+      </c>
+      <c r="M15" s="3">
+        <v>0</v>
+      </c>
+      <c r="N15" s="3">
+        <v>455</v>
+      </c>
+      <c r="O15" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="P15" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q15" s="3" t="s">
+        <v>42</v>
+      </c>
       <c r="R15" s="3"/>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.45">
@@ -1645,4 +1680,123 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0002-000000000000}">
+  <dimension ref="B3:P4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="2.59765625" customWidth="1"/>
+    <col min="2" max="2" width="13.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="16" width="15.59765625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:16" ht="71.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Ally</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="2:16" x14ac:dyDescent="0.45">
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Turret</t>
+        </is>
+      </c>
+      <c r="C4" s="3">
+        <v>100</v>
+      </c>
+      <c r="D4" s="3">
+        <v>300</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3">
+        <v>50</v>
+      </c>
+      <c r="G4" s="3">
+        <v>50</v>
+      </c>
+      <c r="H4" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="I4" s="3">
+        <v>2</v>
+      </c>
+      <c r="J4" s="3">
+        <v>2</v>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>5 / 10</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>0.5 / 1</t>
+        </is>
+      </c>
+      <c r="M4" s="3">
+        <v>25</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Turret</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Khat berserkers now charge and hack with machetes (only within 1 m)
The machete is a real close-quarters weapon: its projectile is "melee" on the
Weapons tab. A berserker sprints at you and swings at 1,200 per minute, but only
hurts you within 1 m. He has a swing animation and sound, and leaves no machete
behind. Kambala Mercenaries now wear 30 armour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CMHq89Xaygpa78Rxcwy3Lr
</commit_message>
<xml_diff>
--- a/data/Game Data.xlsx
+++ b/data/Game Data.xlsx
@@ -1071,7 +1071,7 @@
         <v>100</v>
       </c>
       <c r="D11" s="3">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E11" s="3">
         <v>4</v>
@@ -1871,8 +1871,10 @@
       <c r="O16" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="P16" s="3" t="s">
-        <v>42</v>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>melee</t>
+        </is>
       </c>
       <c r="Q16" s="3" t="s">
         <v>42</v>

</xml_diff>

<commit_message>
Kill streaks: 10 kills earn a mortar strike
Every enemy you kill now counts towards a kill streak (your turret's kills don't).
At 10 kills MORTAR STRIKE AVAILABLE! appears with a mortar-round button; a thin
bar beside the grenade button shows progress. The button puts a laser designator
in your hands (green laser line and dot); SWAP puts it away and keeps the strike;
the button again or FIRE calls it in: INCOMING! 5 s, then 5 shells with white
smoke trails land over 3 s within 8 m of the laser spot (on the roof if it's a
building). They hurt you too. Going down loses the streak. Tune it in
data/killstreaks.csv and the Weapons tab's new Mortar row.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CMHq89Xaygpa78Rxcwy3Lr
</commit_message>
<xml_diff>
--- a/data/Game Data.xlsx
+++ b/data/Game Data.xlsx
@@ -1882,22 +1882,58 @@
       <c r="R16" s="3"/>
     </row>
     <row r="17" spans="2:18" x14ac:dyDescent="0.45">
-      <c r="B17" s="2"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
-      <c r="O17" s="3"/>
-      <c r="P17" s="3"/>
-      <c r="Q17" s="3"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Mortar</t>
+        </is>
+      </c>
+      <c r="C17" s="3">
+        <v>1</v>
+      </c>
+      <c r="D17" s="3">
+        <v>1</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0</v>
+      </c>
+      <c r="F17" s="3">
+        <v>100</v>
+      </c>
+      <c r="G17" s="3">
+        <v>50</v>
+      </c>
+      <c r="H17" s="3">
+        <v>50</v>
+      </c>
+      <c r="I17" s="3">
+        <v>40</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="L17" s="3">
+        <v>0</v>
+      </c>
+      <c r="M17" s="3">
+        <v>0</v>
+      </c>
+      <c r="N17" s="3">
+        <v>15</v>
+      </c>
+      <c r="O17" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>mortar</t>
+        </is>
+      </c>
+      <c r="Q17" s="3" t="s">
+        <v>42</v>
+      </c>
       <c r="R17" s="3"/>
     </row>
     <row r="18" spans="2:18" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
Gunship kill streak (20 kills)
At 20 kills you can call in a gunship: your view goes up to it, circling 150 m
above, through a thermal camera with red squares on enemies and blinking markers
on friendlies. FIRE shoots its 7.62 gun (1,200 a minute, 600 rounds); SWAP
changes to 4 rockets. It leaves after 30 seconds or when both are empty. Its
fire hurts friends too, and your body on the ground can be shot (YOU'RE TAKING
FIRE!); going down ends it. The GUNSHIP TEST button still sends you up for free.

Also: shots from above now hit people through the top of their body.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CMHq89Xaygpa78Rxcwy3Lr
</commit_message>
<xml_diff>
--- a/data/Game Data.xlsx
+++ b/data/Game Data.xlsx
@@ -1937,22 +1937,60 @@
       <c r="R17" s="3"/>
     </row>
     <row r="18" spans="2:18" x14ac:dyDescent="0.45">
-      <c r="B18" s="2"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
-      <c r="N18" s="3"/>
-      <c r="O18" s="3"/>
-      <c r="P18" s="3"/>
-      <c r="Q18" s="3"/>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Gunship gun</t>
+        </is>
+      </c>
+      <c r="C18" s="3">
+        <v>600</v>
+      </c>
+      <c r="D18" s="3">
+        <v>600</v>
+      </c>
+      <c r="E18" s="3">
+        <v>0</v>
+      </c>
+      <c r="F18" s="3">
+        <v>50</v>
+      </c>
+      <c r="G18" s="3">
+        <v>50</v>
+      </c>
+      <c r="H18" s="3">
+        <v>15</v>
+      </c>
+      <c r="I18" s="3">
+        <v>0</v>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="K18" s="3">
+        <v>1200</v>
+      </c>
+      <c r="L18" s="3">
+        <v>0</v>
+      </c>
+      <c r="M18" s="3">
+        <v>5</v>
+      </c>
+      <c r="N18" s="3">
+        <v>420</v>
+      </c>
+      <c r="O18" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="P18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
       <c r="R18" s="3"/>
     </row>
   </sheetData>

</xml_diff>